<commit_message>
report with excel file now can be downloadable
</commit_message>
<xml_diff>
--- a/example_excel_file.xlsx
+++ b/example_excel_file.xlsx
@@ -2,15 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BEstat\BEstat\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{595C280E-DB16-4ADD-9453-0DE53564773B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{595C280E-DB16-4ADD-9453-0DE53564773B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5017B35D-92EF-48AA-9603-3787D8AF4884}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{C3C5C162-4DD9-49EA-AB4D-D6D85BE71FC6}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="14620" xr2:uid="{C3C5C162-4DD9-49EA-AB4D-D6D85BE71FC6}"/>
   </bookViews>
   <sheets>
     <sheet name="PK" sheetId="1" r:id="rId1"/>
@@ -563,16 +558,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC13AB7E-5C38-4EC8-95CB-34D3A5CBBA46}">
   <dimension ref="A1:P21"/>
-  <sheetFormatPr defaultColWidth="8.625" defaultRowHeight="15.75" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.58203125" defaultRowHeight="15" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="8.375" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.33203125" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="7.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.08203125" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="16" width="7.75" style="2" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="8.625" style="2"/>
+    <col min="17" max="16384" width="8.58203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>22</v>
       </c>
@@ -622,7 +617,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
@@ -672,7 +667,7 @@
         <v>0.38</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A3" s="8" t="s">
         <v>1</v>
       </c>
@@ -722,7 +717,7 @@
         <v>0.38800000000000001</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
         <v>2</v>
       </c>
@@ -772,7 +767,7 @@
         <v>0.247</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
         <v>3</v>
       </c>
@@ -822,7 +817,7 @@
         <v>5.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A6" s="8" t="s">
         <v>4</v>
       </c>
@@ -872,7 +867,7 @@
         <v>0.36899999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A7" s="8" t="s">
         <v>5</v>
       </c>
@@ -922,7 +917,7 @@
         <v>0.47299999999999998</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A8" s="8" t="s">
         <v>6</v>
       </c>
@@ -972,7 +967,7 @@
         <v>0.30099999999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
         <v>7</v>
       </c>
@@ -1022,7 +1017,7 @@
         <v>0.434</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>8</v>
       </c>
@@ -1072,7 +1067,7 @@
         <v>0.35699999999999998</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A11" s="8" t="s">
         <v>9</v>
       </c>
@@ -1122,7 +1117,7 @@
         <v>0.34699999999999998</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>10</v>
       </c>
@@ -1172,7 +1167,7 @@
         <v>0.33700000000000002</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>11</v>
       </c>
@@ -1222,7 +1217,7 @@
         <v>0.46400000000000002</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>12</v>
       </c>
@@ -1272,7 +1267,7 @@
         <v>0.222</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>13</v>
       </c>
@@ -1322,7 +1317,7 @@
         <v>8.5999999999999993E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>14</v>
       </c>
@@ -1372,7 +1367,7 @@
         <v>0.32300000000000001</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
         <v>15</v>
       </c>
@@ -1422,7 +1417,7 @@
         <v>0.47899999999999998</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>16</v>
       </c>
@@ -1472,7 +1467,7 @@
         <v>0.315</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
         <v>17</v>
       </c>
@@ -1522,7 +1517,7 @@
         <v>0.29499999999999998</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
         <v>18</v>
       </c>
@@ -1572,7 +1567,7 @@
         <v>0.19700000000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
         <v>19</v>
       </c>
@@ -1625,22 +1620,23 @@
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39B2E545-D7EB-49B6-AAF2-FF6AC2BC07E1}">
   <dimension ref="A1:P21"/>
-  <sheetFormatPr defaultColWidth="8.625" defaultRowHeight="15.75" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.58203125" defaultRowHeight="15" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="8.375" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.33203125" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="7.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.08203125" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="16" width="7.25" style="2" customWidth="1"/>
-    <col min="17" max="16384" width="8.625" style="2"/>
+    <col min="17" max="16384" width="8.58203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>22</v>
       </c>
@@ -1690,7 +1686,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
@@ -1740,7 +1736,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A3" s="8" t="s">
         <v>1</v>
       </c>
@@ -1790,7 +1786,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
         <v>2</v>
       </c>
@@ -1840,7 +1836,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
         <v>3</v>
       </c>
@@ -1890,7 +1886,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A6" s="8" t="s">
         <v>4</v>
       </c>
@@ -1940,7 +1936,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A7" s="8" t="s">
         <v>5</v>
       </c>
@@ -1990,7 +1986,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A8" s="8" t="s">
         <v>6</v>
       </c>
@@ -2040,7 +2036,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
         <v>7</v>
       </c>
@@ -2090,7 +2086,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>8</v>
       </c>
@@ -2140,7 +2136,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A11" s="8" t="s">
         <v>9</v>
       </c>
@@ -2190,7 +2186,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>10</v>
       </c>
@@ -2240,7 +2236,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>11</v>
       </c>
@@ -2290,7 +2286,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>12</v>
       </c>
@@ -2340,7 +2336,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>13</v>
       </c>
@@ -2390,7 +2386,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>14</v>
       </c>
@@ -2440,7 +2436,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
         <v>15</v>
       </c>
@@ -2490,7 +2486,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>16</v>
       </c>
@@ -2540,7 +2536,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
         <v>17</v>
       </c>
@@ -2590,7 +2586,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
         <v>18</v>
       </c>
@@ -2640,7 +2636,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
         <v>19</v>
       </c>
@@ -2693,5 +2689,6 @@
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>